<commit_message>
Sample medicine list: add dummy opening stock, batches, expiry and cost
Opening stock of 5–20 packs, a made-up batch number, an expiry 6–24
months ahead and a cost about 85% of the selling price, so the list can
be imported to try the till straight away.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XWFqcFtqGLbKup45WiLmA8
</commit_message>
<xml_diff>
--- a/samples/Bizflow-medicines-pakistan.xlsx
+++ b/samples/Bizflow-medicines-pakistan.xlsx
@@ -669,10 +669,22 @@
       <c r="V2" t="n">
         <v>20</v>
       </c>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
+      <c r="W2" t="n">
+        <v>80</v>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>PAN-9385</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>07/2027</t>
+        </is>
+      </c>
+      <c r="Z2" t="n">
+        <v>3.36</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -755,10 +767,22 @@
       <c r="V3" t="n">
         <v>20</v>
       </c>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr"/>
+      <c r="W3" t="n">
+        <v>120</v>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>PAN-7891</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>10/2028</t>
+        </is>
+      </c>
+      <c r="Z3" t="n">
+        <v>4.81</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -833,10 +857,22 @@
       <c r="V4" t="n">
         <v>20</v>
       </c>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr"/>
+      <c r="W4" t="n">
+        <v>200</v>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>PAN-8226</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>11/2027</t>
+        </is>
+      </c>
+      <c r="Z4" t="n">
+        <v>5.19</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -903,10 +939,22 @@
       <c r="V5" t="n">
         <v>3</v>
       </c>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="inlineStr"/>
+      <c r="W5" t="n">
+        <v>5</v>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>CAL-2814</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>01/2028</t>
+        </is>
+      </c>
+      <c r="Z5" t="n">
+        <v>128.53</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -973,10 +1021,22 @@
       <c r="V6" t="n">
         <v>3</v>
       </c>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr"/>
+      <c r="W6" t="n">
+        <v>8</v>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>CAL-9032</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>02/2028</t>
+        </is>
+      </c>
+      <c r="Z6" t="n">
+        <v>152.46</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1059,10 +1119,22 @@
       <c r="V7" t="n">
         <v>20</v>
       </c>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
-      <c r="Z7" t="inlineStr"/>
+      <c r="W7" t="n">
+        <v>110</v>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>BRU-6696</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>03/2028</t>
+        </is>
+      </c>
+      <c r="Z7" t="n">
+        <v>4.22</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1129,10 +1201,22 @@
       <c r="V8" t="n">
         <v>3</v>
       </c>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
-      <c r="Y8" t="inlineStr"/>
-      <c r="Z8" t="inlineStr"/>
+      <c r="W8" t="n">
+        <v>17</v>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>BRU-9414</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>06/2027</t>
+        </is>
+      </c>
+      <c r="Z8" t="n">
+        <v>140.8</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1207,10 +1291,22 @@
       <c r="V9" t="n">
         <v>20</v>
       </c>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
-      <c r="Y9" t="inlineStr"/>
-      <c r="Z9" t="inlineStr"/>
+      <c r="W9" t="n">
+        <v>150</v>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>PON-9815</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>01/2028</t>
+        </is>
+      </c>
+      <c r="Z9" t="n">
+        <v>6.19</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1293,10 +1389,22 @@
       <c r="V10" t="n">
         <v>20</v>
       </c>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
-      <c r="Y10" t="inlineStr"/>
-      <c r="Z10" t="inlineStr"/>
+      <c r="W10" t="n">
+        <v>140</v>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>DIS-6062</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>04/2027</t>
+        </is>
+      </c>
+      <c r="Z10" t="n">
+        <v>1.86</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1371,10 +1479,22 @@
       <c r="V11" t="n">
         <v>20</v>
       </c>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
-      <c r="Y11" t="inlineStr"/>
-      <c r="Z11" t="inlineStr"/>
+      <c r="W11" t="n">
+        <v>160</v>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>ARI-7917</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>06/2027</t>
+        </is>
+      </c>
+      <c r="Z11" t="n">
+        <v>10.1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1457,10 +1577,22 @@
       <c r="V12" t="n">
         <v>20</v>
       </c>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
-      <c r="Y12" t="inlineStr"/>
-      <c r="Z12" t="inlineStr"/>
+      <c r="W12" t="n">
+        <v>170</v>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>CAF-9166</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>07/2027</t>
+        </is>
+      </c>
+      <c r="Z12" t="n">
+        <v>11.35</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1543,10 +1675,22 @@
       <c r="V13" t="n">
         <v>20</v>
       </c>
-      <c r="W13" t="inlineStr"/>
-      <c r="X13" t="inlineStr"/>
-      <c r="Y13" t="inlineStr"/>
-      <c r="Z13" t="inlineStr"/>
+      <c r="W13" t="n">
+        <v>180</v>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>DIC-9045</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>04/2028</t>
+        </is>
+      </c>
+      <c r="Z13" t="n">
+        <v>5.95</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1621,10 +1765,22 @@
       <c r="V14" t="n">
         <v>20</v>
       </c>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
-      <c r="Y14" t="inlineStr"/>
-      <c r="Z14" t="inlineStr"/>
+      <c r="W14" t="n">
+        <v>130</v>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>NUB-8851</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>08/2028</t>
+        </is>
+      </c>
+      <c r="Z14" t="n">
+        <v>14.8</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1699,10 +1855,22 @@
       <c r="V15" t="n">
         <v>20</v>
       </c>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
-      <c r="Y15" t="inlineStr"/>
-      <c r="Z15" t="inlineStr"/>
+      <c r="W15" t="n">
+        <v>50</v>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>SYN-3113</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>05/2027</t>
+        </is>
+      </c>
+      <c r="Z15" t="n">
+        <v>19.65</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1769,10 +1937,22 @@
       <c r="V16" t="n">
         <v>3</v>
       </c>
-      <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr"/>
-      <c r="Y16" t="inlineStr"/>
-      <c r="Z16" t="inlineStr"/>
+      <c r="W16" t="n">
+        <v>8</v>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>VOL-8035</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>07/2028</t>
+        </is>
+      </c>
+      <c r="Z16" t="n">
+        <v>362.48</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1847,10 +2027,22 @@
       <c r="V17" t="n">
         <v>12</v>
       </c>
-      <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr"/>
-      <c r="Y17" t="inlineStr"/>
-      <c r="Z17" t="inlineStr"/>
+      <c r="W17" t="n">
+        <v>54</v>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>AUG-4750</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>07/2027</t>
+        </is>
+      </c>
+      <c r="Z17" t="n">
+        <v>63.67</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1925,10 +2117,22 @@
       <c r="V18" t="n">
         <v>12</v>
       </c>
-      <c r="W18" t="inlineStr"/>
-      <c r="X18" t="inlineStr"/>
-      <c r="Y18" t="inlineStr"/>
-      <c r="Z18" t="inlineStr"/>
+      <c r="W18" t="n">
+        <v>114</v>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>AUG-9939</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>12/2027</t>
+        </is>
+      </c>
+      <c r="Z18" t="n">
+        <v>88.91</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1995,10 +2199,22 @@
       <c r="V19" t="n">
         <v>3</v>
       </c>
-      <c r="W19" t="inlineStr"/>
-      <c r="X19" t="inlineStr"/>
-      <c r="Y19" t="inlineStr"/>
-      <c r="Z19" t="inlineStr"/>
+      <c r="W19" t="n">
+        <v>17</v>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>AUG-6040</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>09/2028</t>
+        </is>
+      </c>
+      <c r="Z19" t="n">
+        <v>283.86</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2065,10 +2281,22 @@
       <c r="V20" t="n">
         <v>3</v>
       </c>
-      <c r="W20" t="inlineStr"/>
-      <c r="X20" t="inlineStr"/>
-      <c r="Y20" t="inlineStr"/>
-      <c r="Z20" t="inlineStr"/>
+      <c r="W20" t="n">
+        <v>20</v>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>AUG-7585</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>05/2028</t>
+        </is>
+      </c>
+      <c r="Z20" t="n">
+        <v>364.68</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2151,10 +2379,22 @@
       <c r="V21" t="n">
         <v>20</v>
       </c>
-      <c r="W21" t="inlineStr"/>
-      <c r="X21" t="inlineStr"/>
-      <c r="Y21" t="inlineStr"/>
-      <c r="Z21" t="inlineStr"/>
+      <c r="W21" t="n">
+        <v>110</v>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>AMO-5407</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>04/2027</t>
+        </is>
+      </c>
+      <c r="Z21" t="n">
+        <v>10.05</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2221,10 +2461,22 @@
       <c r="V22" t="n">
         <v>3</v>
       </c>
-      <c r="W22" t="inlineStr"/>
-      <c r="X22" t="inlineStr"/>
-      <c r="Y22" t="inlineStr"/>
-      <c r="Z22" t="inlineStr"/>
+      <c r="W22" t="n">
+        <v>6</v>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>AMO-8507</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>08/2028</t>
+        </is>
+      </c>
+      <c r="Z22" t="n">
+        <v>132.64</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2299,10 +2551,22 @@
       <c r="V23" t="n">
         <v>24</v>
       </c>
-      <c r="W23" t="inlineStr"/>
-      <c r="X23" t="inlineStr"/>
-      <c r="Y23" t="inlineStr"/>
-      <c r="Z23" t="inlineStr"/>
+      <c r="W23" t="n">
+        <v>240</v>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>VEL-4274</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>12/2027</t>
+        </is>
+      </c>
+      <c r="Z23" t="n">
+        <v>26.65</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2369,10 +2633,22 @@
       <c r="V24" t="n">
         <v>3</v>
       </c>
-      <c r="W24" t="inlineStr"/>
-      <c r="X24" t="inlineStr"/>
-      <c r="Y24" t="inlineStr"/>
-      <c r="Z24" t="inlineStr"/>
+      <c r="W24" t="n">
+        <v>20</v>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>VEL-9145</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>05/2028</t>
+        </is>
+      </c>
+      <c r="Z24" t="n">
+        <v>279.84</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2447,10 +2723,22 @@
       <c r="V25" t="n">
         <v>10</v>
       </c>
-      <c r="W25" t="inlineStr"/>
-      <c r="X25" t="inlineStr"/>
-      <c r="Y25" t="inlineStr"/>
-      <c r="Z25" t="inlineStr"/>
+      <c r="W25" t="n">
+        <v>30</v>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>CEF-6188</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>06/2028</t>
+        </is>
+      </c>
+      <c r="Z25" t="n">
+        <v>104.39</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2517,10 +2805,22 @@
       <c r="V26" t="n">
         <v>3</v>
       </c>
-      <c r="W26" t="inlineStr"/>
-      <c r="X26" t="inlineStr"/>
-      <c r="Y26" t="inlineStr"/>
-      <c r="Z26" t="inlineStr"/>
+      <c r="W26" t="n">
+        <v>8</v>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>CEF-9440</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>12/2027</t>
+        </is>
+      </c>
+      <c r="Z26" t="n">
+        <v>313.13</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2595,10 +2895,22 @@
       <c r="V27" t="n">
         <v>20</v>
       </c>
-      <c r="W27" t="inlineStr"/>
-      <c r="X27" t="inlineStr"/>
-      <c r="Y27" t="inlineStr"/>
-      <c r="Z27" t="inlineStr"/>
+      <c r="W27" t="n">
+        <v>190</v>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>NOV-3999</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>05/2028</t>
+        </is>
+      </c>
+      <c r="Z27" t="n">
+        <v>28.01</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2673,10 +2985,22 @@
       <c r="V28" t="n">
         <v>20</v>
       </c>
-      <c r="W28" t="inlineStr"/>
-      <c r="X28" t="inlineStr"/>
-      <c r="Y28" t="inlineStr"/>
-      <c r="Z28" t="inlineStr"/>
+      <c r="W28" t="n">
+        <v>200</v>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>LEF-5365</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>07/2028</t>
+        </is>
+      </c>
+      <c r="Z28" t="n">
+        <v>33.3</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2751,10 +3075,22 @@
       <c r="V29" t="n">
         <v>12</v>
       </c>
-      <c r="W29" t="inlineStr"/>
-      <c r="X29" t="inlineStr"/>
-      <c r="Y29" t="inlineStr"/>
-      <c r="Z29" t="inlineStr"/>
+      <c r="W29" t="n">
+        <v>96</v>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>AZO-7738</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>08/2027</t>
+        </is>
+      </c>
+      <c r="Z29" t="n">
+        <v>61.93</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2821,10 +3157,22 @@
       <c r="V30" t="n">
         <v>3</v>
       </c>
-      <c r="W30" t="inlineStr"/>
-      <c r="X30" t="inlineStr"/>
-      <c r="Y30" t="inlineStr"/>
-      <c r="Z30" t="inlineStr"/>
+      <c r="W30" t="n">
+        <v>19</v>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>AZO-2510</t>
+        </is>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>04/2027</t>
+        </is>
+      </c>
+      <c r="Z30" t="n">
+        <v>236.25</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2899,10 +3247,22 @@
       <c r="V31" t="n">
         <v>20</v>
       </c>
-      <c r="W31" t="inlineStr"/>
-      <c r="X31" t="inlineStr"/>
-      <c r="Y31" t="inlineStr"/>
-      <c r="Z31" t="inlineStr"/>
+      <c r="W31" t="n">
+        <v>190</v>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>KLA-2360</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>10/2027</t>
+        </is>
+      </c>
+      <c r="Z31" t="n">
+        <v>76.94</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2985,10 +3345,22 @@
       <c r="V32" t="n">
         <v>20</v>
       </c>
-      <c r="W32" t="inlineStr"/>
-      <c r="X32" t="inlineStr"/>
-      <c r="Y32" t="inlineStr"/>
-      <c r="Z32" t="inlineStr"/>
+      <c r="W32" t="n">
+        <v>120</v>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>FLA-1731</t>
+        </is>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>09/2028</t>
+        </is>
+      </c>
+      <c r="Z32" t="n">
+        <v>3.72</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3055,10 +3427,22 @@
       <c r="V33" t="n">
         <v>3</v>
       </c>
-      <c r="W33" t="inlineStr"/>
-      <c r="X33" t="inlineStr"/>
-      <c r="Y33" t="inlineStr"/>
-      <c r="Z33" t="inlineStr"/>
+      <c r="W33" t="n">
+        <v>13</v>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>FLA-6853</t>
+        </is>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>08/2027</t>
+        </is>
+      </c>
+      <c r="Z33" t="n">
+        <v>111.81</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3133,10 +3517,22 @@
       <c r="V34" t="n">
         <v>20</v>
       </c>
-      <c r="W34" t="inlineStr"/>
-      <c r="X34" t="inlineStr"/>
-      <c r="Y34" t="inlineStr"/>
-      <c r="Z34" t="inlineStr"/>
+      <c r="W34" t="n">
+        <v>50</v>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>SEP-9060</t>
+        </is>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>08/2027</t>
+        </is>
+      </c>
+      <c r="Z34" t="n">
+        <v>7.97</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3211,10 +3607,22 @@
       <c r="V35" t="n">
         <v>20</v>
       </c>
-      <c r="W35" t="inlineStr"/>
-      <c r="X35" t="inlineStr"/>
-      <c r="Y35" t="inlineStr"/>
-      <c r="Z35" t="inlineStr"/>
+      <c r="W35" t="n">
+        <v>120</v>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>VIB-3149</t>
+        </is>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>08/2028</t>
+        </is>
+      </c>
+      <c r="Z35" t="n">
+        <v>18.66</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3289,10 +3697,22 @@
       <c r="V36" t="n">
         <v>24</v>
       </c>
-      <c r="W36" t="inlineStr"/>
-      <c r="X36" t="inlineStr"/>
-      <c r="Y36" t="inlineStr"/>
-      <c r="Z36" t="inlineStr"/>
+      <c r="W36" t="n">
+        <v>168</v>
+      </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>ERY-3623</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>08/2027</t>
+        </is>
+      </c>
+      <c r="Z36" t="n">
+        <v>20.63</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3367,10 +3787,22 @@
       <c r="V37" t="n">
         <v>16</v>
       </c>
-      <c r="W37" t="inlineStr"/>
-      <c r="X37" t="inlineStr"/>
-      <c r="Y37" t="inlineStr"/>
-      <c r="Z37" t="inlineStr"/>
+      <c r="W37" t="n">
+        <v>112</v>
+      </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>AMP-7396</t>
+        </is>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>08/2027</t>
+        </is>
+      </c>
+      <c r="Z37" t="n">
+        <v>27.64</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3445,10 +3877,22 @@
       <c r="V38" t="n">
         <v>28</v>
       </c>
-      <c r="W38" t="inlineStr"/>
-      <c r="X38" t="inlineStr"/>
-      <c r="Y38" t="inlineStr"/>
-      <c r="Z38" t="inlineStr"/>
+      <c r="W38" t="n">
+        <v>154</v>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>RIS-2738</t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>04/2028</t>
+        </is>
+      </c>
+      <c r="Z38" t="n">
+        <v>22.87</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3523,10 +3967,22 @@
       <c r="V39" t="n">
         <v>28</v>
       </c>
-      <c r="W39" t="inlineStr"/>
-      <c r="X39" t="inlineStr"/>
-      <c r="Y39" t="inlineStr"/>
-      <c r="Z39" t="inlineStr"/>
+      <c r="W39" t="n">
+        <v>98</v>
+      </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>RIS-6685</t>
+        </is>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>03/2028</t>
+        </is>
+      </c>
+      <c r="Z39" t="n">
+        <v>32.92</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3601,10 +4057,22 @@
       <c r="V40" t="n">
         <v>28</v>
       </c>
-      <c r="W40" t="inlineStr"/>
-      <c r="X40" t="inlineStr"/>
-      <c r="Y40" t="inlineStr"/>
-      <c r="Z40" t="inlineStr"/>
+      <c r="W40" t="n">
+        <v>70</v>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>NEX-8799</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>02/2028</t>
+        </is>
+      </c>
+      <c r="Z40" t="n">
+        <v>34.04</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3671,10 +4139,22 @@
       <c r="V41" t="n">
         <v>3</v>
       </c>
-      <c r="W41" t="inlineStr"/>
-      <c r="X41" t="inlineStr"/>
-      <c r="Y41" t="inlineStr"/>
-      <c r="Z41" t="inlineStr"/>
+      <c r="W41" t="n">
+        <v>14</v>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>GAV-2988</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>07/2028</t>
+        </is>
+      </c>
+      <c r="Z41" t="n">
+        <v>287.98</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3741,10 +4221,22 @@
       <c r="V42" t="n">
         <v>3</v>
       </c>
-      <c r="W42" t="inlineStr"/>
-      <c r="X42" t="inlineStr"/>
-      <c r="Y42" t="inlineStr"/>
-      <c r="Z42" t="inlineStr"/>
+      <c r="W42" t="n">
+        <v>19</v>
+      </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>MUC-3797</t>
+        </is>
+      </c>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>08/2027</t>
+        </is>
+      </c>
+      <c r="Z42" t="n">
+        <v>222.12</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3819,10 +4311,22 @@
       <c r="V43" t="n">
         <v>20</v>
       </c>
-      <c r="W43" t="inlineStr"/>
-      <c r="X43" t="inlineStr"/>
-      <c r="Y43" t="inlineStr"/>
-      <c r="Z43" t="inlineStr"/>
+      <c r="W43" t="n">
+        <v>110</v>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>MOT-6511</t>
+        </is>
+      </c>
+      <c r="Y43" t="inlineStr">
+        <is>
+          <t>06/2028</t>
+        </is>
+      </c>
+      <c r="Z43" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3897,10 +4401,22 @@
       <c r="V44" t="n">
         <v>12</v>
       </c>
-      <c r="W44" t="inlineStr"/>
-      <c r="X44" t="inlineStr"/>
-      <c r="Y44" t="inlineStr"/>
-      <c r="Z44" t="inlineStr"/>
+      <c r="W44" t="n">
+        <v>72</v>
+      </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>IMO-2138</t>
+        </is>
+      </c>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>09/2028</t>
+        </is>
+      </c>
+      <c r="Z44" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3975,10 +4491,22 @@
       <c r="V45" t="n">
         <v>20</v>
       </c>
-      <c r="W45" t="inlineStr"/>
-      <c r="X45" t="inlineStr"/>
-      <c r="Y45" t="inlineStr"/>
-      <c r="Z45" t="inlineStr"/>
+      <c r="W45" t="n">
+        <v>170</v>
+      </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>BUS-3840</t>
+        </is>
+      </c>
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>05/2027</t>
+        </is>
+      </c>
+      <c r="Z45" t="n">
+        <v>9.039999999999999</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4053,10 +4581,22 @@
       <c r="V46" t="n">
         <v>20</v>
       </c>
-      <c r="W46" t="inlineStr"/>
-      <c r="X46" t="inlineStr"/>
-      <c r="Y46" t="inlineStr"/>
-      <c r="Z46" t="inlineStr"/>
+      <c r="W46" t="n">
+        <v>60</v>
+      </c>
+      <c r="X46" t="inlineStr">
+        <is>
+          <t>ENT-4088</t>
+        </is>
+      </c>
+      <c r="Y46" t="inlineStr">
+        <is>
+          <t>07/2028</t>
+        </is>
+      </c>
+      <c r="Z46" t="n">
+        <v>7.2</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4131,10 +4671,22 @@
       <c r="V47" t="n">
         <v>20</v>
       </c>
-      <c r="W47" t="inlineStr"/>
-      <c r="X47" t="inlineStr"/>
-      <c r="Y47" t="inlineStr"/>
-      <c r="Z47" t="inlineStr"/>
+      <c r="W47" t="n">
+        <v>50</v>
+      </c>
+      <c r="X47" t="inlineStr">
+        <is>
+          <t>GRA-9682</t>
+        </is>
+      </c>
+      <c r="Y47" t="inlineStr">
+        <is>
+          <t>10/2027</t>
+        </is>
+      </c>
+      <c r="Z47" t="n">
+        <v>4.55</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4201,10 +4753,22 @@
       <c r="V48" t="n">
         <v>3</v>
       </c>
-      <c r="W48" t="inlineStr"/>
-      <c r="X48" t="inlineStr"/>
-      <c r="Y48" t="inlineStr"/>
-      <c r="Z48" t="inlineStr"/>
+      <c r="W48" t="n">
+        <v>9</v>
+      </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>DUP-4047</t>
+        </is>
+      </c>
+      <c r="Y48" t="inlineStr">
+        <is>
+          <t>04/2028</t>
+        </is>
+      </c>
+      <c r="Z48" t="n">
+        <v>464.59</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4279,10 +4843,22 @@
       <c r="V49" t="n">
         <v>20</v>
       </c>
-      <c r="W49" t="inlineStr"/>
-      <c r="X49" t="inlineStr"/>
-      <c r="Y49" t="inlineStr"/>
-      <c r="Z49" t="inlineStr"/>
+      <c r="W49" t="n">
+        <v>130</v>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>DUL-7784</t>
+        </is>
+      </c>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>06/2027</t>
+        </is>
+      </c>
+      <c r="Z49" t="n">
+        <v>7.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4357,10 +4933,22 @@
       <c r="V50" t="n">
         <v>40</v>
       </c>
-      <c r="W50" t="inlineStr"/>
-      <c r="X50" t="inlineStr"/>
-      <c r="Y50" t="inlineStr"/>
-      <c r="Z50" t="inlineStr"/>
+      <c r="W50" t="n">
+        <v>340</v>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>PED-6637</t>
+        </is>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>09/2027</t>
+        </is>
+      </c>
+      <c r="Z50" t="n">
+        <v>25.15</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4435,10 +5023,22 @@
       <c r="V51" t="n">
         <v>12</v>
       </c>
-      <c r="W51" t="inlineStr"/>
-      <c r="X51" t="inlineStr"/>
-      <c r="Y51" t="inlineStr"/>
-      <c r="Z51" t="inlineStr"/>
+      <c r="W51" t="n">
+        <v>78</v>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>ENO-7811</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>01/2028</t>
+        </is>
+      </c>
+      <c r="Z51" t="n">
+        <v>25.44</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4509,10 +5109,22 @@
       <c r="V52" t="n">
         <v>20</v>
       </c>
-      <c r="W52" t="inlineStr"/>
-      <c r="X52" t="inlineStr"/>
-      <c r="Y52" t="inlineStr"/>
-      <c r="Z52" t="inlineStr"/>
+      <c r="W52" t="n">
+        <v>190</v>
+      </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>MAX-9508</t>
+        </is>
+      </c>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>07/2028</t>
+        </is>
+      </c>
+      <c r="Z52" t="n">
+        <v>3.32</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4583,10 +5195,22 @@
       <c r="V53" t="n">
         <v>20</v>
       </c>
-      <c r="W53" t="inlineStr"/>
-      <c r="X53" t="inlineStr"/>
-      <c r="Y53" t="inlineStr"/>
-      <c r="Z53" t="inlineStr"/>
+      <c r="W53" t="n">
+        <v>190</v>
+      </c>
+      <c r="X53" t="inlineStr">
+        <is>
+          <t>SOF-9596</t>
+        </is>
+      </c>
+      <c r="Y53" t="inlineStr">
+        <is>
+          <t>12/2027</t>
+        </is>
+      </c>
+      <c r="Z53" t="n">
+        <v>13.24</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4657,10 +5281,22 @@
       <c r="V54" t="n">
         <v>20</v>
       </c>
-      <c r="W54" t="inlineStr"/>
-      <c r="X54" t="inlineStr"/>
-      <c r="Y54" t="inlineStr"/>
-      <c r="Z54" t="inlineStr"/>
+      <c r="W54" t="n">
+        <v>80</v>
+      </c>
+      <c r="X54" t="inlineStr">
+        <is>
+          <t>RIG-4790</t>
+        </is>
+      </c>
+      <c r="Y54" t="inlineStr">
+        <is>
+          <t>04/2027</t>
+        </is>
+      </c>
+      <c r="Z54" t="n">
+        <v>6.1</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4735,10 +5371,22 @@
       <c r="V55" t="n">
         <v>20</v>
       </c>
-      <c r="W55" t="inlineStr"/>
-      <c r="X55" t="inlineStr"/>
-      <c r="Y55" t="inlineStr"/>
-      <c r="Z55" t="inlineStr"/>
+      <c r="W55" t="n">
+        <v>70</v>
+      </c>
+      <c r="X55" t="inlineStr">
+        <is>
+          <t>TEL-6413</t>
+        </is>
+      </c>
+      <c r="Y55" t="inlineStr">
+        <is>
+          <t>05/2028</t>
+        </is>
+      </c>
+      <c r="Z55" t="n">
+        <v>27.93</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4813,10 +5461,22 @@
       <c r="V56" t="n">
         <v>20</v>
       </c>
-      <c r="W56" t="inlineStr"/>
-      <c r="X56" t="inlineStr"/>
-      <c r="Y56" t="inlineStr"/>
-      <c r="Z56" t="inlineStr"/>
+      <c r="W56" t="n">
+        <v>100</v>
+      </c>
+      <c r="X56" t="inlineStr">
+        <is>
+          <t>TEL-6766</t>
+        </is>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>09/2027</t>
+        </is>
+      </c>
+      <c r="Z56" t="n">
+        <v>36.86</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4891,10 +5551,22 @@
       <c r="V57" t="n">
         <v>20</v>
       </c>
-      <c r="W57" t="inlineStr"/>
-      <c r="X57" t="inlineStr"/>
-      <c r="Y57" t="inlineStr"/>
-      <c r="Z57" t="inlineStr"/>
+      <c r="W57" t="n">
+        <v>160</v>
+      </c>
+      <c r="X57" t="inlineStr">
+        <is>
+          <t>AVI-9820</t>
+        </is>
+      </c>
+      <c r="Y57" t="inlineStr">
+        <is>
+          <t>10/2027</t>
+        </is>
+      </c>
+      <c r="Z57" t="n">
+        <v>2.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4961,10 +5633,22 @@
       <c r="V58" t="n">
         <v>3</v>
       </c>
-      <c r="W58" t="inlineStr"/>
-      <c r="X58" t="inlineStr"/>
-      <c r="Y58" t="inlineStr"/>
-      <c r="Z58" t="inlineStr"/>
+      <c r="W58" t="n">
+        <v>8</v>
+      </c>
+      <c r="X58" t="inlineStr">
+        <is>
+          <t>HYD-5595</t>
+        </is>
+      </c>
+      <c r="Y58" t="inlineStr">
+        <is>
+          <t>09/2028</t>
+        </is>
+      </c>
+      <c r="Z58" t="n">
+        <v>128.59</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5027,10 +5711,22 @@
       <c r="V59" t="n">
         <v>3</v>
       </c>
-      <c r="W59" t="inlineStr"/>
-      <c r="X59" t="inlineStr"/>
-      <c r="Y59" t="inlineStr"/>
-      <c r="Z59" t="inlineStr"/>
+      <c r="W59" t="n">
+        <v>11</v>
+      </c>
+      <c r="X59" t="inlineStr">
+        <is>
+          <t>ACE-5392</t>
+        </is>
+      </c>
+      <c r="Y59" t="inlineStr">
+        <is>
+          <t>09/2028</t>
+        </is>
+      </c>
+      <c r="Z59" t="n">
+        <v>119.59</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5105,10 +5801,22 @@
       <c r="V60" t="n">
         <v>16</v>
       </c>
-      <c r="W60" t="inlineStr"/>
-      <c r="X60" t="inlineStr"/>
-      <c r="Y60" t="inlineStr"/>
-      <c r="Z60" t="inlineStr"/>
+      <c r="W60" t="n">
+        <v>72</v>
+      </c>
+      <c r="X60" t="inlineStr">
+        <is>
+          <t>STR-5320</t>
+        </is>
+      </c>
+      <c r="Y60" t="inlineStr">
+        <is>
+          <t>07/2027</t>
+        </is>
+      </c>
+      <c r="Z60" t="n">
+        <v>14.46</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5175,10 +5883,22 @@
       <c r="V61" t="n">
         <v>3</v>
       </c>
-      <c r="W61" t="inlineStr"/>
-      <c r="X61" t="inlineStr"/>
-      <c r="Y61" t="inlineStr"/>
-      <c r="Z61" t="inlineStr"/>
+      <c r="W61" t="n">
+        <v>18</v>
+      </c>
+      <c r="X61" t="inlineStr">
+        <is>
+          <t>OTR-1990</t>
+        </is>
+      </c>
+      <c r="Y61" t="inlineStr">
+        <is>
+          <t>03/2028</t>
+        </is>
+      </c>
+      <c r="Z61" t="n">
+        <v>157.75</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5245,10 +5965,22 @@
       <c r="V62" t="n">
         <v>3</v>
       </c>
-      <c r="W62" t="inlineStr"/>
-      <c r="X62" t="inlineStr"/>
-      <c r="Y62" t="inlineStr"/>
-      <c r="Z62" t="inlineStr"/>
+      <c r="W62" t="n">
+        <v>10</v>
+      </c>
+      <c r="X62" t="inlineStr">
+        <is>
+          <t>VIC-2741</t>
+        </is>
+      </c>
+      <c r="Y62" t="inlineStr">
+        <is>
+          <t>08/2028</t>
+        </is>
+      </c>
+      <c r="Z62" t="n">
+        <v>240.45</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -5315,10 +6047,22 @@
       <c r="V63" t="n">
         <v>3</v>
       </c>
-      <c r="W63" t="inlineStr"/>
-      <c r="X63" t="inlineStr"/>
-      <c r="Y63" t="inlineStr"/>
-      <c r="Z63" t="inlineStr"/>
+      <c r="W63" t="n">
+        <v>15</v>
+      </c>
+      <c r="X63" t="inlineStr">
+        <is>
+          <t>VEN-2047</t>
+        </is>
+      </c>
+      <c r="Y63" t="inlineStr">
+        <is>
+          <t>01/2028</t>
+        </is>
+      </c>
+      <c r="Z63" t="n">
+        <v>418.3</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5385,10 +6129,22 @@
       <c r="V64" t="n">
         <v>3</v>
       </c>
-      <c r="W64" t="inlineStr"/>
-      <c r="X64" t="inlineStr"/>
-      <c r="Y64" t="inlineStr"/>
-      <c r="Z64" t="inlineStr"/>
+      <c r="W64" t="n">
+        <v>15</v>
+      </c>
+      <c r="X64" t="inlineStr">
+        <is>
+          <t>VEN-5196</t>
+        </is>
+      </c>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>06/2027</t>
+        </is>
+      </c>
+      <c r="Z64" t="n">
+        <v>78.81999999999999</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5455,10 +6211,22 @@
       <c r="V65" t="n">
         <v>3</v>
       </c>
-      <c r="W65" t="inlineStr"/>
-      <c r="X65" t="inlineStr"/>
-      <c r="Y65" t="inlineStr"/>
-      <c r="Z65" t="inlineStr"/>
+      <c r="W65" t="n">
+        <v>5</v>
+      </c>
+      <c r="X65" t="inlineStr">
+        <is>
+          <t>SER-5211</t>
+        </is>
+      </c>
+      <c r="Y65" t="inlineStr">
+        <is>
+          <t>05/2028</t>
+        </is>
+      </c>
+      <c r="Z65" t="n">
+        <v>1647.16</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5533,10 +6301,22 @@
       <c r="V66" t="n">
         <v>28</v>
       </c>
-      <c r="W66" t="inlineStr"/>
-      <c r="X66" t="inlineStr"/>
-      <c r="Y66" t="inlineStr"/>
-      <c r="Z66" t="inlineStr"/>
+      <c r="W66" t="n">
+        <v>70</v>
+      </c>
+      <c r="X66" t="inlineStr">
+        <is>
+          <t>SIN-4853</t>
+        </is>
+      </c>
+      <c r="Y66" t="inlineStr">
+        <is>
+          <t>04/2027</t>
+        </is>
+      </c>
+      <c r="Z66" t="n">
+        <v>45.88</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5611,10 +6391,22 @@
       <c r="V67" t="n">
         <v>28</v>
       </c>
-      <c r="W67" t="inlineStr"/>
-      <c r="X67" t="inlineStr"/>
-      <c r="Y67" t="inlineStr"/>
-      <c r="Z67" t="inlineStr"/>
+      <c r="W67" t="n">
+        <v>196</v>
+      </c>
+      <c r="X67" t="inlineStr">
+        <is>
+          <t>MYT-6739</t>
+        </is>
+      </c>
+      <c r="Y67" t="inlineStr">
+        <is>
+          <t>02/2028</t>
+        </is>
+      </c>
+      <c r="Z67" t="n">
+        <v>27.78</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5697,10 +6489,22 @@
       <c r="V68" t="n">
         <v>20</v>
       </c>
-      <c r="W68" t="inlineStr"/>
-      <c r="X68" t="inlineStr"/>
-      <c r="Y68" t="inlineStr"/>
-      <c r="Z68" t="inlineStr"/>
+      <c r="W68" t="n">
+        <v>190</v>
+      </c>
+      <c r="X68" t="inlineStr">
+        <is>
+          <t>GLU-1622</t>
+        </is>
+      </c>
+      <c r="Y68" t="inlineStr">
+        <is>
+          <t>04/2028</t>
+        </is>
+      </c>
+      <c r="Z68" t="n">
+        <v>3.94</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5783,10 +6587,22 @@
       <c r="V69" t="n">
         <v>20</v>
       </c>
-      <c r="W69" t="inlineStr"/>
-      <c r="X69" t="inlineStr"/>
-      <c r="Y69" t="inlineStr"/>
-      <c r="Z69" t="inlineStr"/>
+      <c r="W69" t="n">
+        <v>150</v>
+      </c>
+      <c r="X69" t="inlineStr">
+        <is>
+          <t>GLU-8580</t>
+        </is>
+      </c>
+      <c r="Y69" t="inlineStr">
+        <is>
+          <t>05/2028</t>
+        </is>
+      </c>
+      <c r="Z69" t="n">
+        <v>5.31</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5869,10 +6685,22 @@
       <c r="V70" t="n">
         <v>20</v>
       </c>
-      <c r="W70" t="inlineStr"/>
-      <c r="X70" t="inlineStr"/>
-      <c r="Y70" t="inlineStr"/>
-      <c r="Z70" t="inlineStr"/>
+      <c r="W70" t="n">
+        <v>80</v>
+      </c>
+      <c r="X70" t="inlineStr">
+        <is>
+          <t>AMA-9212</t>
+        </is>
+      </c>
+      <c r="Y70" t="inlineStr">
+        <is>
+          <t>12/2027</t>
+        </is>
+      </c>
+      <c r="Z70" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5947,10 +6775,22 @@
       <c r="V71" t="n">
         <v>20</v>
       </c>
-      <c r="W71" t="inlineStr"/>
-      <c r="X71" t="inlineStr"/>
-      <c r="Y71" t="inlineStr"/>
-      <c r="Z71" t="inlineStr"/>
+      <c r="W71" t="n">
+        <v>170</v>
+      </c>
+      <c r="X71" t="inlineStr">
+        <is>
+          <t>DAO-6837</t>
+        </is>
+      </c>
+      <c r="Y71" t="inlineStr">
+        <is>
+          <t>05/2027</t>
+        </is>
+      </c>
+      <c r="Z71" t="n">
+        <v>4.02</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -6025,10 +6865,22 @@
       <c r="V72" t="n">
         <v>28</v>
       </c>
-      <c r="W72" t="inlineStr"/>
-      <c r="X72" t="inlineStr"/>
-      <c r="Y72" t="inlineStr"/>
-      <c r="Z72" t="inlineStr"/>
+      <c r="W72" t="n">
+        <v>252</v>
+      </c>
+      <c r="X72" t="inlineStr">
+        <is>
+          <t>JAN-5610</t>
+        </is>
+      </c>
+      <c r="Y72" t="inlineStr">
+        <is>
+          <t>02/2028</t>
+        </is>
+      </c>
+      <c r="Z72" t="n">
+        <v>90.39</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -6111,10 +6963,22 @@
       <c r="V73" t="n">
         <v>28</v>
       </c>
-      <c r="W73" t="inlineStr"/>
-      <c r="X73" t="inlineStr"/>
-      <c r="Y73" t="inlineStr"/>
-      <c r="Z73" t="inlineStr"/>
+      <c r="W73" t="n">
+        <v>196</v>
+      </c>
+      <c r="X73" t="inlineStr">
+        <is>
+          <t>GAL-3004</t>
+        </is>
+      </c>
+      <c r="Y73" t="inlineStr">
+        <is>
+          <t>01/2028</t>
+        </is>
+      </c>
+      <c r="Z73" t="n">
+        <v>43.18</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -6197,10 +7061,22 @@
       <c r="V74" t="n">
         <v>20</v>
       </c>
-      <c r="W74" t="inlineStr"/>
-      <c r="X74" t="inlineStr"/>
-      <c r="Y74" t="inlineStr"/>
-      <c r="Z74" t="inlineStr"/>
+      <c r="W74" t="n">
+        <v>180</v>
+      </c>
+      <c r="X74" t="inlineStr">
+        <is>
+          <t>CON-1332</t>
+        </is>
+      </c>
+      <c r="Y74" t="inlineStr">
+        <is>
+          <t>09/2028</t>
+        </is>
+      </c>
+      <c r="Z74" t="n">
+        <v>12.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -6283,10 +7159,22 @@
       <c r="V75" t="n">
         <v>28</v>
       </c>
-      <c r="W75" t="inlineStr"/>
-      <c r="X75" t="inlineStr"/>
-      <c r="Y75" t="inlineStr"/>
-      <c r="Z75" t="inlineStr"/>
+      <c r="W75" t="n">
+        <v>210</v>
+      </c>
+      <c r="X75" t="inlineStr">
+        <is>
+          <t>TEN-1919</t>
+        </is>
+      </c>
+      <c r="Y75" t="inlineStr">
+        <is>
+          <t>07/2027</t>
+        </is>
+      </c>
+      <c r="Z75" t="n">
+        <v>8.32</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -6369,10 +7257,22 @@
       <c r="V76" t="n">
         <v>20</v>
       </c>
-      <c r="W76" t="inlineStr"/>
-      <c r="X76" t="inlineStr"/>
-      <c r="Y76" t="inlineStr"/>
-      <c r="Z76" t="inlineStr"/>
+      <c r="W76" t="n">
+        <v>100</v>
+      </c>
+      <c r="X76" t="inlineStr">
+        <is>
+          <t>NOR-2937</t>
+        </is>
+      </c>
+      <c r="Y76" t="inlineStr">
+        <is>
+          <t>05/2027</t>
+        </is>
+      </c>
+      <c r="Z76" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -6447,10 +7347,22 @@
       <c r="V77" t="n">
         <v>28</v>
       </c>
-      <c r="W77" t="inlineStr"/>
-      <c r="X77" t="inlineStr"/>
-      <c r="Y77" t="inlineStr"/>
-      <c r="Z77" t="inlineStr"/>
+      <c r="W77" t="n">
+        <v>126</v>
+      </c>
+      <c r="X77" t="inlineStr">
+        <is>
+          <t>COZ-5951</t>
+        </is>
+      </c>
+      <c r="Y77" t="inlineStr">
+        <is>
+          <t>04/2027</t>
+        </is>
+      </c>
+      <c r="Z77" t="n">
+        <v>26.76</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6533,10 +7445,22 @@
       <c r="V78" t="n">
         <v>20</v>
       </c>
-      <c r="W78" t="inlineStr"/>
-      <c r="X78" t="inlineStr"/>
-      <c r="Y78" t="inlineStr"/>
-      <c r="Z78" t="inlineStr"/>
+      <c r="W78" t="n">
+        <v>180</v>
+      </c>
+      <c r="X78" t="inlineStr">
+        <is>
+          <t>COV-6832</t>
+        </is>
+      </c>
+      <c r="Y78" t="inlineStr">
+        <is>
+          <t>05/2028</t>
+        </is>
+      </c>
+      <c r="Z78" t="n">
+        <v>27.35</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6611,10 +7535,22 @@
       <c r="V79" t="n">
         <v>20</v>
       </c>
-      <c r="W79" t="inlineStr"/>
-      <c r="X79" t="inlineStr"/>
-      <c r="Y79" t="inlineStr"/>
-      <c r="Z79" t="inlineStr"/>
+      <c r="W79" t="n">
+        <v>170</v>
+      </c>
+      <c r="X79" t="inlineStr">
+        <is>
+          <t>LAS-7897</t>
+        </is>
+      </c>
+      <c r="Y79" t="inlineStr">
+        <is>
+          <t>11/2027</t>
+        </is>
+      </c>
+      <c r="Z79" t="n">
+        <v>4.63</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6697,10 +7633,22 @@
       <c r="V80" t="n">
         <v>20</v>
       </c>
-      <c r="W80" t="inlineStr"/>
-      <c r="X80" t="inlineStr"/>
-      <c r="Y80" t="inlineStr"/>
-      <c r="Z80" t="inlineStr"/>
+      <c r="W80" t="n">
+        <v>90</v>
+      </c>
+      <c r="X80" t="inlineStr">
+        <is>
+          <t>ALD-1465</t>
+        </is>
+      </c>
+      <c r="Y80" t="inlineStr">
+        <is>
+          <t>09/2028</t>
+        </is>
+      </c>
+      <c r="Z80" t="n">
+        <v>10.8</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -6771,10 +7719,22 @@
       <c r="V81" t="n">
         <v>20</v>
       </c>
-      <c r="W81" t="inlineStr"/>
-      <c r="X81" t="inlineStr"/>
-      <c r="Y81" t="inlineStr"/>
-      <c r="Z81" t="inlineStr"/>
+      <c r="W81" t="n">
+        <v>170</v>
+      </c>
+      <c r="X81" t="inlineStr">
+        <is>
+          <t>LOW-3419</t>
+        </is>
+      </c>
+      <c r="Y81" t="inlineStr">
+        <is>
+          <t>11/2027</t>
+        </is>
+      </c>
+      <c r="Z81" t="n">
+        <v>22.71</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6857,10 +7817,22 @@
       <c r="V82" t="n">
         <v>20</v>
       </c>
-      <c r="W82" t="inlineStr"/>
-      <c r="X82" t="inlineStr"/>
-      <c r="Y82" t="inlineStr"/>
-      <c r="Z82" t="inlineStr"/>
+      <c r="W82" t="n">
+        <v>50</v>
+      </c>
+      <c r="X82" t="inlineStr">
+        <is>
+          <t>LOP-9866</t>
+        </is>
+      </c>
+      <c r="Y82" t="inlineStr">
+        <is>
+          <t>07/2028</t>
+        </is>
+      </c>
+      <c r="Z82" t="n">
+        <v>2.87</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -6935,10 +7907,22 @@
       <c r="V83" t="n">
         <v>20</v>
       </c>
-      <c r="W83" t="inlineStr"/>
-      <c r="X83" t="inlineStr"/>
-      <c r="Y83" t="inlineStr"/>
-      <c r="Z83" t="inlineStr"/>
+      <c r="W83" t="n">
+        <v>180</v>
+      </c>
+      <c r="X83" t="inlineStr">
+        <is>
+          <t>LIP-6156</t>
+        </is>
+      </c>
+      <c r="Y83" t="inlineStr">
+        <is>
+          <t>08/2027</t>
+        </is>
+      </c>
+      <c r="Z83" t="n">
+        <v>17.55</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -7013,10 +7997,22 @@
       <c r="V84" t="n">
         <v>20</v>
       </c>
-      <c r="W84" t="inlineStr"/>
-      <c r="X84" t="inlineStr"/>
-      <c r="Y84" t="inlineStr"/>
-      <c r="Z84" t="inlineStr"/>
+      <c r="W84" t="n">
+        <v>70</v>
+      </c>
+      <c r="X84" t="inlineStr">
+        <is>
+          <t>LIP-1622</t>
+        </is>
+      </c>
+      <c r="Y84" t="inlineStr">
+        <is>
+          <t>08/2028</t>
+        </is>
+      </c>
+      <c r="Z84" t="n">
+        <v>41.78</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -7091,10 +8087,22 @@
       <c r="V85" t="n">
         <v>20</v>
       </c>
-      <c r="W85" t="inlineStr"/>
-      <c r="X85" t="inlineStr"/>
-      <c r="Y85" t="inlineStr"/>
-      <c r="Z85" t="inlineStr"/>
+      <c r="W85" t="n">
+        <v>130</v>
+      </c>
+      <c r="X85" t="inlineStr">
+        <is>
+          <t>CAC-9527</t>
+        </is>
+      </c>
+      <c r="Y85" t="inlineStr">
+        <is>
+          <t>02/2028</t>
+        </is>
+      </c>
+      <c r="Z85" t="n">
+        <v>33.62</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7169,10 +8177,22 @@
       <c r="V86" t="n">
         <v>60</v>
       </c>
-      <c r="W86" t="inlineStr"/>
-      <c r="X86" t="inlineStr"/>
-      <c r="Y86" t="inlineStr"/>
-      <c r="Z86" t="inlineStr"/>
+      <c r="W86" t="n">
+        <v>180</v>
+      </c>
+      <c r="X86" t="inlineStr">
+        <is>
+          <t>SUR-1186</t>
+        </is>
+      </c>
+      <c r="Y86" t="inlineStr">
+        <is>
+          <t>11/2027</t>
+        </is>
+      </c>
+      <c r="Z86" t="n">
+        <v>19.48</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -7255,10 +8275,22 @@
       <c r="V87" t="n">
         <v>20</v>
       </c>
-      <c r="W87" t="inlineStr"/>
-      <c r="X87" t="inlineStr"/>
-      <c r="Y87" t="inlineStr"/>
-      <c r="Z87" t="inlineStr"/>
+      <c r="W87" t="n">
+        <v>200</v>
+      </c>
+      <c r="X87" t="inlineStr">
+        <is>
+          <t>NEU-4634</t>
+        </is>
+      </c>
+      <c r="Y87" t="inlineStr">
+        <is>
+          <t>08/2028</t>
+        </is>
+      </c>
+      <c r="Z87" t="n">
+        <v>11.53</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -7333,10 +8365,22 @@
       <c r="V88" t="n">
         <v>60</v>
       </c>
-      <c r="W88" t="inlineStr"/>
-      <c r="X88" t="inlineStr"/>
-      <c r="Y88" t="inlineStr"/>
-      <c r="Z88" t="inlineStr"/>
+      <c r="W88" t="n">
+        <v>270</v>
+      </c>
+      <c r="X88" t="inlineStr">
+        <is>
+          <t>IBE-7538</t>
+        </is>
+      </c>
+      <c r="Y88" t="inlineStr">
+        <is>
+          <t>03/2028</t>
+        </is>
+      </c>
+      <c r="Z88" t="n">
+        <v>19.85</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -7419,10 +8463,22 @@
       <c r="V89" t="n">
         <v>20</v>
       </c>
-      <c r="W89" t="inlineStr"/>
-      <c r="X89" t="inlineStr"/>
-      <c r="Y89" t="inlineStr"/>
-      <c r="Z89" t="inlineStr"/>
+      <c r="W89" t="n">
+        <v>120</v>
+      </c>
+      <c r="X89" t="inlineStr">
+        <is>
+          <t>SAN-5518</t>
+        </is>
+      </c>
+      <c r="Y89" t="inlineStr">
+        <is>
+          <t>02/2028</t>
+        </is>
+      </c>
+      <c r="Z89" t="n">
+        <v>19.63</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -7505,10 +8561,22 @@
       <c r="V90" t="n">
         <v>20</v>
       </c>
-      <c r="W90" t="inlineStr"/>
-      <c r="X90" t="inlineStr"/>
-      <c r="Y90" t="inlineStr"/>
-      <c r="Z90" t="inlineStr"/>
+      <c r="W90" t="n">
+        <v>110</v>
+      </c>
+      <c r="X90" t="inlineStr">
+        <is>
+          <t>EVI-8524</t>
+        </is>
+      </c>
+      <c r="Y90" t="inlineStr">
+        <is>
+          <t>06/2028</t>
+        </is>
+      </c>
+      <c r="Z90" t="n">
+        <v>26.96</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -7587,10 +8655,22 @@
       <c r="V91" t="n">
         <v>20</v>
       </c>
-      <c r="W91" t="inlineStr"/>
-      <c r="X91" t="inlineStr"/>
-      <c r="Y91" t="inlineStr"/>
-      <c r="Z91" t="inlineStr"/>
+      <c r="W91" t="n">
+        <v>200</v>
+      </c>
+      <c r="X91" t="inlineStr">
+        <is>
+          <t>FOL-6114</t>
+        </is>
+      </c>
+      <c r="Y91" t="inlineStr">
+        <is>
+          <t>10/2027</t>
+        </is>
+      </c>
+      <c r="Z91" t="n">
+        <v>1.31</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -7653,10 +8733,22 @@
       <c r="V92" t="n">
         <v>3</v>
       </c>
-      <c r="W92" t="inlineStr"/>
-      <c r="X92" t="inlineStr"/>
-      <c r="Y92" t="inlineStr"/>
-      <c r="Z92" t="inlineStr"/>
+      <c r="W92" t="n">
+        <v>10</v>
+      </c>
+      <c r="X92" t="inlineStr">
+        <is>
+          <t>VIT-3519</t>
+        </is>
+      </c>
+      <c r="Y92" t="inlineStr">
+        <is>
+          <t>07/2028</t>
+        </is>
+      </c>
+      <c r="Z92" t="n">
+        <v>197.27</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -7731,10 +8823,22 @@
       <c r="V93" t="n">
         <v>60</v>
       </c>
-      <c r="W93" t="inlineStr"/>
-      <c r="X93" t="inlineStr"/>
-      <c r="Y93" t="inlineStr"/>
-      <c r="Z93" t="inlineStr"/>
+      <c r="W93" t="n">
+        <v>150</v>
+      </c>
+      <c r="X93" t="inlineStr">
+        <is>
+          <t>CEN-9572</t>
+        </is>
+      </c>
+      <c r="Y93" t="inlineStr">
+        <is>
+          <t>05/2028</t>
+        </is>
+      </c>
+      <c r="Z93" t="n">
+        <v>48.24</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -7813,10 +8917,22 @@
       <c r="V94" t="n">
         <v>20</v>
       </c>
-      <c r="W94" t="inlineStr"/>
-      <c r="X94" t="inlineStr"/>
-      <c r="Y94" t="inlineStr"/>
-      <c r="Z94" t="inlineStr"/>
+      <c r="W94" t="n">
+        <v>60</v>
+      </c>
+      <c r="X94" t="inlineStr">
+        <is>
+          <t>QAL-2379</t>
+        </is>
+      </c>
+      <c r="Y94" t="inlineStr">
+        <is>
+          <t>01/2028</t>
+        </is>
+      </c>
+      <c r="Z94" t="n">
+        <v>12.02</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -7891,10 +9007,22 @@
       <c r="V95" t="n">
         <v>200</v>
       </c>
-      <c r="W95" t="inlineStr"/>
-      <c r="X95" t="inlineStr"/>
-      <c r="Y95" t="inlineStr"/>
-      <c r="Z95" t="inlineStr"/>
+      <c r="W95" t="n">
+        <v>1600</v>
+      </c>
+      <c r="X95" t="inlineStr">
+        <is>
+          <t>ELT-5342</t>
+        </is>
+      </c>
+      <c r="Y95" t="inlineStr">
+        <is>
+          <t>08/2027</t>
+        </is>
+      </c>
+      <c r="Z95" t="n">
+        <v>1.96</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -7969,10 +9097,22 @@
       <c r="V96" t="n">
         <v>20</v>
       </c>
-      <c r="W96" t="inlineStr"/>
-      <c r="X96" t="inlineStr"/>
-      <c r="Y96" t="inlineStr"/>
-      <c r="Z96" t="inlineStr"/>
+      <c r="W96" t="n">
+        <v>80</v>
+      </c>
+      <c r="X96" t="inlineStr">
+        <is>
+          <t>DEL-1300</t>
+        </is>
+      </c>
+      <c r="Y96" t="inlineStr">
+        <is>
+          <t>09/2028</t>
+        </is>
+      </c>
+      <c r="Z96" t="n">
+        <v>3.08</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -8047,10 +9187,22 @@
       <c r="V97" t="n">
         <v>40</v>
       </c>
-      <c r="W97" t="inlineStr"/>
-      <c r="X97" t="inlineStr"/>
-      <c r="Y97" t="inlineStr"/>
-      <c r="Z97" t="inlineStr"/>
+      <c r="W97" t="n">
+        <v>220</v>
+      </c>
+      <c r="X97" t="inlineStr">
+        <is>
+          <t>DUP-6025</t>
+        </is>
+      </c>
+      <c r="Y97" t="inlineStr">
+        <is>
+          <t>10/2028</t>
+        </is>
+      </c>
+      <c r="Z97" t="n">
+        <v>58.79</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -8117,10 +9269,22 @@
       <c r="V98" t="n">
         <v>3</v>
       </c>
-      <c r="W98" t="inlineStr"/>
-      <c r="X98" t="inlineStr"/>
-      <c r="Y98" t="inlineStr"/>
-      <c r="Z98" t="inlineStr"/>
+      <c r="W98" t="n">
+        <v>6</v>
+      </c>
+      <c r="X98" t="inlineStr">
+        <is>
+          <t>DIF-7235</t>
+        </is>
+      </c>
+      <c r="Y98" t="inlineStr">
+        <is>
+          <t>09/2028</t>
+        </is>
+      </c>
+      <c r="Z98" t="n">
+        <v>307.07</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -8187,10 +9351,22 @@
       <c r="V99" t="n">
         <v>3</v>
       </c>
-      <c r="W99" t="inlineStr"/>
-      <c r="X99" t="inlineStr"/>
-      <c r="Y99" t="inlineStr"/>
-      <c r="Z99" t="inlineStr"/>
+      <c r="W99" t="n">
+        <v>10</v>
+      </c>
+      <c r="X99" t="inlineStr">
+        <is>
+          <t>CAN-2719</t>
+        </is>
+      </c>
+      <c r="Y99" t="inlineStr">
+        <is>
+          <t>06/2027</t>
+        </is>
+      </c>
+      <c r="Z99" t="n">
+        <v>403.84</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -8257,10 +9433,22 @@
       <c r="V100" t="n">
         <v>3</v>
       </c>
-      <c r="W100" t="inlineStr"/>
-      <c r="X100" t="inlineStr"/>
-      <c r="Y100" t="inlineStr"/>
-      <c r="Z100" t="inlineStr"/>
+      <c r="W100" t="n">
+        <v>9</v>
+      </c>
+      <c r="X100" t="inlineStr">
+        <is>
+          <t>ZEN-6465</t>
+        </is>
+      </c>
+      <c r="Y100" t="inlineStr">
+        <is>
+          <t>09/2028</t>
+        </is>
+      </c>
+      <c r="Z100" t="n">
+        <v>69.12</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -8327,10 +9515,22 @@
       <c r="V101" t="n">
         <v>3</v>
       </c>
-      <c r="W101" t="inlineStr"/>
-      <c r="X101" t="inlineStr"/>
-      <c r="Y101" t="inlineStr"/>
-      <c r="Z101" t="inlineStr"/>
+      <c r="W101" t="n">
+        <v>13</v>
+      </c>
+      <c r="X101" t="inlineStr">
+        <is>
+          <t>POL-4109</t>
+        </is>
+      </c>
+      <c r="Y101" t="inlineStr">
+        <is>
+          <t>09/2027</t>
+        </is>
+      </c>
+      <c r="Z101" t="n">
+        <v>226.43</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -8397,10 +9597,22 @@
       <c r="V102" t="n">
         <v>3</v>
       </c>
-      <c r="W102" t="inlineStr"/>
-      <c r="X102" t="inlineStr"/>
-      <c r="Y102" t="inlineStr"/>
-      <c r="Z102" t="inlineStr"/>
+      <c r="W102" t="n">
+        <v>14</v>
+      </c>
+      <c r="X102" t="inlineStr">
+        <is>
+          <t>FUC-5678</t>
+        </is>
+      </c>
+      <c r="Y102" t="inlineStr">
+        <is>
+          <t>03/2028</t>
+        </is>
+      </c>
+      <c r="Z102" t="n">
+        <v>410.48</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -8467,10 +9679,22 @@
       <c r="V103" t="n">
         <v>3</v>
       </c>
-      <c r="W103" t="inlineStr"/>
-      <c r="X103" t="inlineStr"/>
-      <c r="Y103" t="inlineStr"/>
-      <c r="Z103" t="inlineStr"/>
+      <c r="W103" t="n">
+        <v>9</v>
+      </c>
+      <c r="X103" t="inlineStr">
+        <is>
+          <t>BET-4091</t>
+        </is>
+      </c>
+      <c r="Y103" t="inlineStr">
+        <is>
+          <t>04/2027</t>
+        </is>
+      </c>
+      <c r="Z103" t="n">
+        <v>158.11</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -8537,10 +9761,22 @@
       <c r="V104" t="n">
         <v>3</v>
       </c>
-      <c r="W104" t="inlineStr"/>
-      <c r="X104" t="inlineStr"/>
-      <c r="Y104" t="inlineStr"/>
-      <c r="Z104" t="inlineStr"/>
+      <c r="W104" t="n">
+        <v>20</v>
+      </c>
+      <c r="X104" t="inlineStr">
+        <is>
+          <t>TOB-6827</t>
+        </is>
+      </c>
+      <c r="Y104" t="inlineStr">
+        <is>
+          <t>09/2028</t>
+        </is>
+      </c>
+      <c r="Z104" t="n">
+        <v>403.12</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -8607,10 +9843,22 @@
       <c r="V105" t="n">
         <v>3</v>
       </c>
-      <c r="W105" t="inlineStr"/>
-      <c r="X105" t="inlineStr"/>
-      <c r="Y105" t="inlineStr"/>
-      <c r="Z105" t="inlineStr"/>
+      <c r="W105" t="n">
+        <v>10</v>
+      </c>
+      <c r="X105" t="inlineStr">
+        <is>
+          <t>OTO-1483</t>
+        </is>
+      </c>
+      <c r="Y105" t="inlineStr">
+        <is>
+          <t>09/2027</t>
+        </is>
+      </c>
+      <c r="Z105" t="n">
+        <v>224.46</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -8677,10 +9925,22 @@
       <c r="V106" t="n">
         <v>3</v>
       </c>
-      <c r="W106" t="inlineStr"/>
-      <c r="X106" t="inlineStr"/>
-      <c r="Y106" t="inlineStr"/>
-      <c r="Z106" t="inlineStr"/>
+      <c r="W106" t="n">
+        <v>15</v>
+      </c>
+      <c r="X106" t="inlineStr">
+        <is>
+          <t>PYO-3685</t>
+        </is>
+      </c>
+      <c r="Y106" t="inlineStr">
+        <is>
+          <t>04/2027</t>
+        </is>
+      </c>
+      <c r="Z106" t="n">
+        <v>136.38</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -8747,10 +10007,22 @@
       <c r="V107" t="n">
         <v>3</v>
       </c>
-      <c r="W107" t="inlineStr"/>
-      <c r="X107" t="inlineStr"/>
-      <c r="Y107" t="inlineStr"/>
-      <c r="Z107" t="inlineStr"/>
+      <c r="W107" t="n">
+        <v>8</v>
+      </c>
+      <c r="X107" t="inlineStr">
+        <is>
+          <t>DET-1032</t>
+        </is>
+      </c>
+      <c r="Y107" t="inlineStr">
+        <is>
+          <t>03/2028</t>
+        </is>
+      </c>
+      <c r="Z107" t="n">
+        <v>357.38</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -8813,10 +10085,22 @@
       <c r="V108" t="n">
         <v>3</v>
       </c>
-      <c r="W108" t="inlineStr"/>
-      <c r="X108" t="inlineStr"/>
-      <c r="Y108" t="inlineStr"/>
-      <c r="Z108" t="inlineStr"/>
+      <c r="W108" t="n">
+        <v>7</v>
+      </c>
+      <c r="X108" t="inlineStr">
+        <is>
+          <t>SAV-4542</t>
+        </is>
+      </c>
+      <c r="Y108" t="inlineStr">
+        <is>
+          <t>09/2028</t>
+        </is>
+      </c>
+      <c r="Z108" t="n">
+        <v>303.15</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -8883,10 +10167,22 @@
       <c r="V109" t="n">
         <v>3</v>
       </c>
-      <c r="W109" t="inlineStr"/>
-      <c r="X109" t="inlineStr"/>
-      <c r="Y109" t="inlineStr"/>
-      <c r="Z109" t="inlineStr"/>
+      <c r="W109" t="n">
+        <v>9</v>
+      </c>
+      <c r="X109" t="inlineStr">
+        <is>
+          <t>WOO-5065</t>
+        </is>
+      </c>
+      <c r="Y109" t="inlineStr">
+        <is>
+          <t>08/2027</t>
+        </is>
+      </c>
+      <c r="Z109" t="n">
+        <v>188.31</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8899,7 +10195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -8935,36 +10231,43 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Barcodes, rack, opening stock, batch, expiry and cost are left empty on purpose:</t>
+          <t>OPENING STOCK, BATCH NO, EXPIRY AND COST ARE DUMMY VALUES for trying the app.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>stock comes in through Purchases (with batch and expiry), and barcodes are best scanned from the pack in the product form.</t>
+          <t>For a real shop, replace them with what is on your shelves (or clear them and receive stock through Purchases).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Where the company is blank, the maker was not certain; fill it in from the pack.</t>
+          <t>Barcodes and rack are left empty: barcodes are best scanned from the pack in the product form.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Where the company is blank, the maker was not certain; fill it in from the pack.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Medicines are set to 0% sales tax.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-    </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>To import: Backoffice &gt; Inventory &gt; Import from Excel &gt; choose this file. The "Products" sheet is read.</t>
         </is>

</xml_diff>

<commit_message>
Sample medicine list: add dummy barcodes, barcode pack and racks
Valid EAN-13 barcodes in the 2… range GS1 keeps for in-store codes (so
they never clash with a real pack), each on the product's largest pack,
and a rack letter per category. Price per kg stays empty: all are sold
by the pack.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XWFqcFtqGLbKup45WiLmA8
</commit_message>
<xml_diff>
--- a/samples/Bizflow-medicines-pakistan.xlsx
+++ b/samples/Bizflow-medicines-pakistan.xlsx
@@ -655,9 +655,21 @@
         <v>800</v>
       </c>
       <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>2042600000019</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
       <c r="T2" t="n">
         <v>0</v>
       </c>
@@ -753,9 +765,21 @@
         <v>660</v>
       </c>
       <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>2042600000026</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
       <c r="T3" t="n">
         <v>0</v>
       </c>
@@ -843,9 +867,21 @@
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2042600000033</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
       <c r="T4" t="n">
         <v>0</v>
       </c>
@@ -925,9 +961,21 @@
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2042600000040</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Btl</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
       <c r="T5" t="n">
         <v>0</v>
       </c>
@@ -1007,9 +1055,21 @@
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>2042600000057</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Btl</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
       <c r="T6" t="n">
         <v>0</v>
       </c>
@@ -1105,9 +1165,21 @@
         <v>150</v>
       </c>
       <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>2042600000064</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
       <c r="T7" t="n">
         <v>0</v>
       </c>
@@ -1187,9 +1259,21 @@
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>2042600000071</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Btl</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
       <c r="T8" t="n">
         <v>0</v>
       </c>
@@ -1277,9 +1361,21 @@
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>2042600000088</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
       <c r="T9" t="n">
         <v>0</v>
       </c>
@@ -1375,9 +1471,21 @@
         <v>440</v>
       </c>
       <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>2042600000095</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
       <c r="T10" t="n">
         <v>0</v>
       </c>
@@ -1465,9 +1573,21 @@
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>2042600000101</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
       <c r="T11" t="n">
         <v>0</v>
       </c>
@@ -1563,9 +1683,21 @@
         <v>260</v>
       </c>
       <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>2042600000118</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
       <c r="T12" t="n">
         <v>0</v>
       </c>
@@ -1661,9 +1793,21 @@
         <v>140</v>
       </c>
       <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
-      <c r="S13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>2042600000125</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
       <c r="T13" t="n">
         <v>0</v>
       </c>
@@ -1751,9 +1895,21 @@
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>2042600000132</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
       <c r="T14" t="n">
         <v>0</v>
       </c>
@@ -1841,9 +1997,21 @@
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
-      <c r="S15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>2042600000149</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
       <c r="T15" t="n">
         <v>0</v>
       </c>
@@ -1923,9 +2091,21 @@
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>2042600000156</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Tube</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
       <c r="T16" t="n">
         <v>0</v>
       </c>
@@ -2013,9 +2193,21 @@
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>2042600000163</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
       <c r="T17" t="n">
         <v>0</v>
       </c>
@@ -2103,9 +2295,21 @@
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>2042600000170</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
       <c r="T18" t="n">
         <v>0</v>
       </c>
@@ -2185,9 +2389,21 @@
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>2042600000187</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Btl</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
       <c r="T19" t="n">
         <v>0</v>
       </c>
@@ -2267,9 +2483,21 @@
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>2042600000194</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Btl</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
       <c r="T20" t="n">
         <v>0</v>
       </c>
@@ -2365,9 +2593,21 @@
         <v>240</v>
       </c>
       <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>2042600000200</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
       <c r="T21" t="n">
         <v>0</v>
       </c>
@@ -2447,9 +2687,21 @@
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
-      <c r="S22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>2042600000217</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Btl</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
       <c r="T22" t="n">
         <v>0</v>
       </c>
@@ -2537,9 +2789,21 @@
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>2042600000224</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
       <c r="T23" t="n">
         <v>0</v>
       </c>
@@ -2619,9 +2883,21 @@
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>2042600000231</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Btl</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
       <c r="T24" t="n">
         <v>0</v>
       </c>
@@ -2709,9 +2985,21 @@
       <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>2042600000248</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
       <c r="T25" t="n">
         <v>0</v>
       </c>
@@ -2791,9 +3079,21 @@
       <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr"/>
-      <c r="S26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>2042600000255</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Btl</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
       <c r="T26" t="n">
         <v>0</v>
       </c>
@@ -2881,9 +3181,21 @@
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
-      <c r="S27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>2042600000262</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
       <c r="T27" t="n">
         <v>0</v>
       </c>
@@ -2971,9 +3283,21 @@
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr"/>
-      <c r="S28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>2042600000279</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
       <c r="T28" t="n">
         <v>0</v>
       </c>
@@ -3061,9 +3385,21 @@
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr"/>
-      <c r="S29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>2042600000286</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
       <c r="T29" t="n">
         <v>0</v>
       </c>
@@ -3143,9 +3479,21 @@
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr"/>
-      <c r="S30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>2042600000293</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Btl</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
       <c r="T30" t="n">
         <v>0</v>
       </c>
@@ -3233,9 +3581,21 @@
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>2042600000309</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
       <c r="T31" t="n">
         <v>0</v>
       </c>
@@ -3331,9 +3691,21 @@
         <v>900</v>
       </c>
       <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>2042600000316</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
       <c r="T32" t="n">
         <v>0</v>
       </c>
@@ -3413,9 +3785,21 @@
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr"/>
-      <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr"/>
-      <c r="S33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>2042600000323</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Btl</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
       <c r="T33" t="n">
         <v>0</v>
       </c>
@@ -3503,9 +3887,21 @@
       <c r="N34" t="inlineStr"/>
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="inlineStr"/>
-      <c r="S34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>2042600000330</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
       <c r="T34" t="n">
         <v>0</v>
       </c>
@@ -3593,9 +3989,21 @@
       <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="inlineStr"/>
-      <c r="S35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>2042600000347</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
       <c r="T35" t="n">
         <v>0</v>
       </c>
@@ -3683,9 +4091,21 @@
       <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr"/>
-      <c r="S36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>2042600000354</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
       <c r="T36" t="n">
         <v>0</v>
       </c>
@@ -3773,9 +4193,21 @@
       <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
-      <c r="R37" t="inlineStr"/>
-      <c r="S37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>2042600000361</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
       <c r="T37" t="n">
         <v>0</v>
       </c>
@@ -3863,9 +4295,21 @@
       <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="inlineStr"/>
-      <c r="S38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>2042600000378</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
       <c r="T38" t="n">
         <v>0</v>
       </c>
@@ -3953,9 +4397,21 @@
       <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
-      <c r="R39" t="inlineStr"/>
-      <c r="S39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>2042600000385</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
       <c r="T39" t="n">
         <v>0</v>
       </c>
@@ -4043,9 +4499,21 @@
       <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
-      <c r="R40" t="inlineStr"/>
-      <c r="S40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>2042600000392</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
       <c r="T40" t="n">
         <v>0</v>
       </c>
@@ -4125,9 +4593,21 @@
       <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="inlineStr"/>
-      <c r="S41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>2042600000408</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Btl</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
       <c r="T41" t="n">
         <v>0</v>
       </c>
@@ -4207,9 +4687,21 @@
       <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr"/>
-      <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="inlineStr"/>
-      <c r="S42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>2042600000415</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Btl</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
       <c r="T42" t="n">
         <v>0</v>
       </c>
@@ -4297,9 +4789,21 @@
       <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr"/>
-      <c r="Q43" t="inlineStr"/>
-      <c r="R43" t="inlineStr"/>
-      <c r="S43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>2042600000422</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
       <c r="T43" t="n">
         <v>0</v>
       </c>
@@ -4387,9 +4891,21 @@
       <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr"/>
-      <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="inlineStr"/>
-      <c r="S44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>2042600000439</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
       <c r="T44" t="n">
         <v>0</v>
       </c>
@@ -4477,9 +4993,21 @@
       <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr"/>
-      <c r="Q45" t="inlineStr"/>
-      <c r="R45" t="inlineStr"/>
-      <c r="S45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>2042600000446</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
       <c r="T45" t="n">
         <v>0</v>
       </c>
@@ -4567,9 +5095,21 @@
       <c r="N46" t="inlineStr"/>
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr"/>
-      <c r="Q46" t="inlineStr"/>
-      <c r="R46" t="inlineStr"/>
-      <c r="S46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>2042600000453</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
       <c r="T46" t="n">
         <v>0</v>
       </c>
@@ -4657,9 +5197,21 @@
       <c r="N47" t="inlineStr"/>
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr"/>
-      <c r="Q47" t="inlineStr"/>
-      <c r="R47" t="inlineStr"/>
-      <c r="S47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>2042600000460</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
       <c r="T47" t="n">
         <v>0</v>
       </c>
@@ -4739,9 +5291,21 @@
       <c r="N48" t="inlineStr"/>
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr"/>
-      <c r="Q48" t="inlineStr"/>
-      <c r="R48" t="inlineStr"/>
-      <c r="S48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>2042600000477</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>Btl</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
       <c r="T48" t="n">
         <v>0</v>
       </c>
@@ -4829,9 +5393,21 @@
       <c r="N49" t="inlineStr"/>
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr"/>
-      <c r="Q49" t="inlineStr"/>
-      <c r="R49" t="inlineStr"/>
-      <c r="S49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>2042600000484</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
       <c r="T49" t="n">
         <v>0</v>
       </c>
@@ -4919,9 +5495,21 @@
       <c r="N50" t="inlineStr"/>
       <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr"/>
-      <c r="Q50" t="inlineStr"/>
-      <c r="R50" t="inlineStr"/>
-      <c r="S50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>2042600000491</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
       <c r="T50" t="n">
         <v>0</v>
       </c>
@@ -5009,9 +5597,21 @@
       <c r="N51" t="inlineStr"/>
       <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr"/>
-      <c r="Q51" t="inlineStr"/>
-      <c r="R51" t="inlineStr"/>
-      <c r="S51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>2042600000507</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
       <c r="T51" t="n">
         <v>0</v>
       </c>
@@ -5095,9 +5695,21 @@
       <c r="N52" t="inlineStr"/>
       <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr"/>
-      <c r="R52" t="inlineStr"/>
-      <c r="S52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>2042600000514</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
       <c r="T52" t="n">
         <v>0</v>
       </c>
@@ -5181,9 +5793,21 @@
       <c r="N53" t="inlineStr"/>
       <c r="O53" t="inlineStr"/>
       <c r="P53" t="inlineStr"/>
-      <c r="Q53" t="inlineStr"/>
-      <c r="R53" t="inlineStr"/>
-      <c r="S53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>2042600000521</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
       <c r="T53" t="n">
         <v>0</v>
       </c>
@@ -5267,9 +5891,21 @@
       <c r="N54" t="inlineStr"/>
       <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr"/>
-      <c r="Q54" t="inlineStr"/>
-      <c r="R54" t="inlineStr"/>
-      <c r="S54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>2042600000538</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
       <c r="T54" t="n">
         <v>0</v>
       </c>
@@ -5357,9 +5993,21 @@
       <c r="N55" t="inlineStr"/>
       <c r="O55" t="inlineStr"/>
       <c r="P55" t="inlineStr"/>
-      <c r="Q55" t="inlineStr"/>
-      <c r="R55" t="inlineStr"/>
-      <c r="S55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>2042600000545</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
       <c r="T55" t="n">
         <v>0</v>
       </c>
@@ -5447,9 +6095,21 @@
       <c r="N56" t="inlineStr"/>
       <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr"/>
-      <c r="Q56" t="inlineStr"/>
-      <c r="R56" t="inlineStr"/>
-      <c r="S56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>2042600000552</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
       <c r="T56" t="n">
         <v>0</v>
       </c>
@@ -5537,9 +6197,21 @@
       <c r="N57" t="inlineStr"/>
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr"/>
-      <c r="Q57" t="inlineStr"/>
-      <c r="R57" t="inlineStr"/>
-      <c r="S57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>2042600000569</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
       <c r="T57" t="n">
         <v>0</v>
       </c>
@@ -5619,9 +6291,21 @@
       <c r="N58" t="inlineStr"/>
       <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr"/>
-      <c r="Q58" t="inlineStr"/>
-      <c r="R58" t="inlineStr"/>
-      <c r="S58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>2042600000576</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>Btl</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
       <c r="T58" t="n">
         <v>0</v>
       </c>
@@ -5697,9 +6381,21 @@
       <c r="N59" t="inlineStr"/>
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr"/>
-      <c r="Q59" t="inlineStr"/>
-      <c r="R59" t="inlineStr"/>
-      <c r="S59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>2042600000583</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>Btl</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
       <c r="T59" t="n">
         <v>0</v>
       </c>
@@ -5787,9 +6483,21 @@
       <c r="N60" t="inlineStr"/>
       <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr"/>
-      <c r="Q60" t="inlineStr"/>
-      <c r="R60" t="inlineStr"/>
-      <c r="S60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>2042600000590</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
       <c r="T60" t="n">
         <v>0</v>
       </c>
@@ -5869,9 +6577,21 @@
       <c r="N61" t="inlineStr"/>
       <c r="O61" t="inlineStr"/>
       <c r="P61" t="inlineStr"/>
-      <c r="Q61" t="inlineStr"/>
-      <c r="R61" t="inlineStr"/>
-      <c r="S61" t="inlineStr"/>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>2042600000606</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Btl</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
       <c r="T61" t="n">
         <v>0</v>
       </c>
@@ -5951,9 +6671,21 @@
       <c r="N62" t="inlineStr"/>
       <c r="O62" t="inlineStr"/>
       <c r="P62" t="inlineStr"/>
-      <c r="Q62" t="inlineStr"/>
-      <c r="R62" t="inlineStr"/>
-      <c r="S62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>2042600000613</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>Jar</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
       <c r="T62" t="n">
         <v>0</v>
       </c>
@@ -6033,9 +6765,21 @@
       <c r="N63" t="inlineStr"/>
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr"/>
-      <c r="Q63" t="inlineStr"/>
-      <c r="R63" t="inlineStr"/>
-      <c r="S63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>2042600000620</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>Pc</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
       <c r="T63" t="n">
         <v>0</v>
       </c>
@@ -6115,9 +6859,21 @@
       <c r="N64" t="inlineStr"/>
       <c r="O64" t="inlineStr"/>
       <c r="P64" t="inlineStr"/>
-      <c r="Q64" t="inlineStr"/>
-      <c r="R64" t="inlineStr"/>
-      <c r="S64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>2042600000637</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>Btl</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
       <c r="T64" t="n">
         <v>0</v>
       </c>
@@ -6197,9 +6953,21 @@
       <c r="N65" t="inlineStr"/>
       <c r="O65" t="inlineStr"/>
       <c r="P65" t="inlineStr"/>
-      <c r="Q65" t="inlineStr"/>
-      <c r="R65" t="inlineStr"/>
-      <c r="S65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>2042600000644</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>Pc</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
       <c r="T65" t="n">
         <v>0</v>
       </c>
@@ -6287,9 +7055,21 @@
       <c r="N66" t="inlineStr"/>
       <c r="O66" t="inlineStr"/>
       <c r="P66" t="inlineStr"/>
-      <c r="Q66" t="inlineStr"/>
-      <c r="R66" t="inlineStr"/>
-      <c r="S66" t="inlineStr"/>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>2042600000651</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>E4</t>
+        </is>
+      </c>
       <c r="T66" t="n">
         <v>0</v>
       </c>
@@ -6377,9 +7157,21 @@
       <c r="N67" t="inlineStr"/>
       <c r="O67" t="inlineStr"/>
       <c r="P67" t="inlineStr"/>
-      <c r="Q67" t="inlineStr"/>
-      <c r="R67" t="inlineStr"/>
-      <c r="S67" t="inlineStr"/>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>2042600000668</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
       <c r="T67" t="n">
         <v>0</v>
       </c>
@@ -6475,9 +7267,21 @@
         <v>230</v>
       </c>
       <c r="P68" t="inlineStr"/>
-      <c r="Q68" t="inlineStr"/>
-      <c r="R68" t="inlineStr"/>
-      <c r="S68" t="inlineStr"/>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>2042600000675</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="T68" t="n">
         <v>0</v>
       </c>
@@ -6573,9 +7377,21 @@
         <v>310</v>
       </c>
       <c r="P69" t="inlineStr"/>
-      <c r="Q69" t="inlineStr"/>
-      <c r="R69" t="inlineStr"/>
-      <c r="S69" t="inlineStr"/>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>2042600000682</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
       <c r="T69" t="n">
         <v>0</v>
       </c>
@@ -6671,9 +7487,21 @@
         <v>520</v>
       </c>
       <c r="P70" t="inlineStr"/>
-      <c r="Q70" t="inlineStr"/>
-      <c r="R70" t="inlineStr"/>
-      <c r="S70" t="inlineStr"/>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>2042600000699</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
       <c r="T70" t="n">
         <v>0</v>
       </c>
@@ -6761,9 +7589,21 @@
       <c r="N71" t="inlineStr"/>
       <c r="O71" t="inlineStr"/>
       <c r="P71" t="inlineStr"/>
-      <c r="Q71" t="inlineStr"/>
-      <c r="R71" t="inlineStr"/>
-      <c r="S71" t="inlineStr"/>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>2042600000705</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
       <c r="T71" t="n">
         <v>0</v>
       </c>
@@ -6851,9 +7691,21 @@
       <c r="N72" t="inlineStr"/>
       <c r="O72" t="inlineStr"/>
       <c r="P72" t="inlineStr"/>
-      <c r="Q72" t="inlineStr"/>
-      <c r="R72" t="inlineStr"/>
-      <c r="S72" t="inlineStr"/>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>2042600000712</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="T72" t="n">
         <v>0</v>
       </c>
@@ -6949,9 +7801,21 @@
         <v>1400</v>
       </c>
       <c r="P73" t="inlineStr"/>
-      <c r="Q73" t="inlineStr"/>
-      <c r="R73" t="inlineStr"/>
-      <c r="S73" t="inlineStr"/>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>2042600000729</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
       <c r="T73" t="n">
         <v>0</v>
       </c>
@@ -7047,9 +7911,21 @@
         <v>450</v>
       </c>
       <c r="P74" t="inlineStr"/>
-      <c r="Q74" t="inlineStr"/>
-      <c r="R74" t="inlineStr"/>
-      <c r="S74" t="inlineStr"/>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>2042600000736</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
       <c r="T74" t="n">
         <v>0</v>
       </c>
@@ -7145,9 +8021,21 @@
         <v>280</v>
       </c>
       <c r="P75" t="inlineStr"/>
-      <c r="Q75" t="inlineStr"/>
-      <c r="R75" t="inlineStr"/>
-      <c r="S75" t="inlineStr"/>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>2042600000743</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>G2</t>
+        </is>
+      </c>
       <c r="T75" t="n">
         <v>0</v>
       </c>
@@ -7243,9 +8131,21 @@
         <v>520</v>
       </c>
       <c r="P76" t="inlineStr"/>
-      <c r="Q76" t="inlineStr"/>
-      <c r="R76" t="inlineStr"/>
-      <c r="S76" t="inlineStr"/>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>2042600000750</t>
+        </is>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
       <c r="T76" t="n">
         <v>0</v>
       </c>
@@ -7333,9 +8233,21 @@
       <c r="N77" t="inlineStr"/>
       <c r="O77" t="inlineStr"/>
       <c r="P77" t="inlineStr"/>
-      <c r="Q77" t="inlineStr"/>
-      <c r="R77" t="inlineStr"/>
-      <c r="S77" t="inlineStr"/>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>2042600000767</t>
+        </is>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>G4</t>
+        </is>
+      </c>
       <c r="T77" t="n">
         <v>0</v>
       </c>
@@ -7431,9 +8343,21 @@
         <v>960</v>
       </c>
       <c r="P78" t="inlineStr"/>
-      <c r="Q78" t="inlineStr"/>
-      <c r="R78" t="inlineStr"/>
-      <c r="S78" t="inlineStr"/>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>2042600000774</t>
+        </is>
+      </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
       <c r="T78" t="n">
         <v>0</v>
       </c>
@@ -7521,9 +8445,21 @@
       <c r="N79" t="inlineStr"/>
       <c r="O79" t="inlineStr"/>
       <c r="P79" t="inlineStr"/>
-      <c r="Q79" t="inlineStr"/>
-      <c r="R79" t="inlineStr"/>
-      <c r="S79" t="inlineStr"/>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>2042600000781</t>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>G2</t>
+        </is>
+      </c>
       <c r="T79" t="n">
         <v>0</v>
       </c>
@@ -7619,9 +8555,21 @@
         <v>260</v>
       </c>
       <c r="P80" t="inlineStr"/>
-      <c r="Q80" t="inlineStr"/>
-      <c r="R80" t="inlineStr"/>
-      <c r="S80" t="inlineStr"/>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>2042600000798</t>
+        </is>
+      </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
       <c r="T80" t="n">
         <v>0</v>
       </c>
@@ -7705,9 +8653,21 @@
       <c r="N81" t="inlineStr"/>
       <c r="O81" t="inlineStr"/>
       <c r="P81" t="inlineStr"/>
-      <c r="Q81" t="inlineStr"/>
-      <c r="R81" t="inlineStr"/>
-      <c r="S81" t="inlineStr"/>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>2042600000804</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>G4</t>
+        </is>
+      </c>
       <c r="T81" t="n">
         <v>0</v>
       </c>
@@ -7803,9 +8763,21 @@
         <v>105</v>
       </c>
       <c r="P82" t="inlineStr"/>
-      <c r="Q82" t="inlineStr"/>
-      <c r="R82" t="inlineStr"/>
-      <c r="S82" t="inlineStr"/>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>2042600000811</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
       <c r="T82" t="n">
         <v>0</v>
       </c>
@@ -7893,9 +8865,21 @@
       <c r="N83" t="inlineStr"/>
       <c r="O83" t="inlineStr"/>
       <c r="P83" t="inlineStr"/>
-      <c r="Q83" t="inlineStr"/>
-      <c r="R83" t="inlineStr"/>
-      <c r="S83" t="inlineStr"/>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>2042600000828</t>
+        </is>
+      </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S83" t="inlineStr">
+        <is>
+          <t>G2</t>
+        </is>
+      </c>
       <c r="T83" t="n">
         <v>0</v>
       </c>
@@ -7983,9 +8967,21 @@
       <c r="N84" t="inlineStr"/>
       <c r="O84" t="inlineStr"/>
       <c r="P84" t="inlineStr"/>
-      <c r="Q84" t="inlineStr"/>
-      <c r="R84" t="inlineStr"/>
-      <c r="S84" t="inlineStr"/>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>2042600000835</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
       <c r="T84" t="n">
         <v>0</v>
       </c>
@@ -8073,9 +9069,21 @@
       <c r="N85" t="inlineStr"/>
       <c r="O85" t="inlineStr"/>
       <c r="P85" t="inlineStr"/>
-      <c r="Q85" t="inlineStr"/>
-      <c r="R85" t="inlineStr"/>
-      <c r="S85" t="inlineStr"/>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>2042600000842</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>Tube</t>
+        </is>
+      </c>
+      <c r="S85" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
       <c r="T85" t="n">
         <v>0</v>
       </c>
@@ -8163,9 +9171,21 @@
       <c r="N86" t="inlineStr"/>
       <c r="O86" t="inlineStr"/>
       <c r="P86" t="inlineStr"/>
-      <c r="Q86" t="inlineStr"/>
-      <c r="R86" t="inlineStr"/>
-      <c r="S86" t="inlineStr"/>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>2042600000859</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>Bottle</t>
+        </is>
+      </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>H2</t>
+        </is>
+      </c>
       <c r="T86" t="n">
         <v>0</v>
       </c>
@@ -8261,9 +9281,21 @@
         <v>420</v>
       </c>
       <c r="P87" t="inlineStr"/>
-      <c r="Q87" t="inlineStr"/>
-      <c r="R87" t="inlineStr"/>
-      <c r="S87" t="inlineStr"/>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>2042600000866</t>
+        </is>
+      </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S87" t="inlineStr">
+        <is>
+          <t>H3</t>
+        </is>
+      </c>
       <c r="T87" t="n">
         <v>0</v>
       </c>
@@ -8351,9 +9383,21 @@
       <c r="N88" t="inlineStr"/>
       <c r="O88" t="inlineStr"/>
       <c r="P88" t="inlineStr"/>
-      <c r="Q88" t="inlineStr"/>
-      <c r="R88" t="inlineStr"/>
-      <c r="S88" t="inlineStr"/>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>2042600000873</t>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>Bottle</t>
+        </is>
+      </c>
+      <c r="S88" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
       <c r="T88" t="n">
         <v>0</v>
       </c>
@@ -8449,9 +9493,21 @@
         <v>460</v>
       </c>
       <c r="P89" t="inlineStr"/>
-      <c r="Q89" t="inlineStr"/>
-      <c r="R89" t="inlineStr"/>
-      <c r="S89" t="inlineStr"/>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>2042600000880</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
       <c r="T89" t="n">
         <v>0</v>
       </c>
@@ -8547,9 +9603,21 @@
         <v>960</v>
       </c>
       <c r="P90" t="inlineStr"/>
-      <c r="Q90" t="inlineStr"/>
-      <c r="R90" t="inlineStr"/>
-      <c r="S90" t="inlineStr"/>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>2042600000897</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>H2</t>
+        </is>
+      </c>
       <c r="T90" t="n">
         <v>0</v>
       </c>
@@ -8641,9 +9709,21 @@
         <v>150</v>
       </c>
       <c r="P91" t="inlineStr"/>
-      <c r="Q91" t="inlineStr"/>
-      <c r="R91" t="inlineStr"/>
-      <c r="S91" t="inlineStr"/>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>2042600000903</t>
+        </is>
+      </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t>H3</t>
+        </is>
+      </c>
       <c r="T91" t="n">
         <v>0</v>
       </c>
@@ -8719,9 +9799,21 @@
       <c r="N92" t="inlineStr"/>
       <c r="O92" t="inlineStr"/>
       <c r="P92" t="inlineStr"/>
-      <c r="Q92" t="inlineStr"/>
-      <c r="R92" t="inlineStr"/>
-      <c r="S92" t="inlineStr"/>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>2042600000910</t>
+        </is>
+      </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>Cap</t>
+        </is>
+      </c>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
       <c r="T92" t="n">
         <v>0</v>
       </c>
@@ -8809,9 +9901,21 @@
       <c r="N93" t="inlineStr"/>
       <c r="O93" t="inlineStr"/>
       <c r="P93" t="inlineStr"/>
-      <c r="Q93" t="inlineStr"/>
-      <c r="R93" t="inlineStr"/>
-      <c r="S93" t="inlineStr"/>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>2042600000927</t>
+        </is>
+      </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>Bottle</t>
+        </is>
+      </c>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
       <c r="T93" t="n">
         <v>0</v>
       </c>
@@ -8903,9 +10007,21 @@
         <v>420</v>
       </c>
       <c r="P94" t="inlineStr"/>
-      <c r="Q94" t="inlineStr"/>
-      <c r="R94" t="inlineStr"/>
-      <c r="S94" t="inlineStr"/>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>2042600000934</t>
+        </is>
+      </c>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="S94" t="inlineStr">
+        <is>
+          <t>H2</t>
+        </is>
+      </c>
       <c r="T94" t="n">
         <v>0</v>
       </c>
@@ -8993,9 +10109,21 @@
       <c r="N95" t="inlineStr"/>
       <c r="O95" t="inlineStr"/>
       <c r="P95" t="inlineStr"/>
-      <c r="Q95" t="inlineStr"/>
-      <c r="R95" t="inlineStr"/>
-      <c r="S95" t="inlineStr"/>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>2042600000941</t>
+        </is>
+      </c>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>Bottle</t>
+        </is>
+      </c>
+      <c r="S95" t="inlineStr">
+        <is>
+          <t>I1</t>
+        </is>
+      </c>
       <c r="T95" t="n">
         <v>0</v>
       </c>
@@ -9083,9 +10211,21 @@
       <c r="N96" t="inlineStr"/>
       <c r="O96" t="inlineStr"/>
       <c r="P96" t="inlineStr"/>
-      <c r="Q96" t="inlineStr"/>
-      <c r="R96" t="inlineStr"/>
-      <c r="S96" t="inlineStr"/>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>2042600000958</t>
+        </is>
+      </c>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S96" t="inlineStr">
+        <is>
+          <t>I2</t>
+        </is>
+      </c>
       <c r="T96" t="n">
         <v>0</v>
       </c>
@@ -9173,9 +10313,21 @@
       <c r="N97" t="inlineStr"/>
       <c r="O97" t="inlineStr"/>
       <c r="P97" t="inlineStr"/>
-      <c r="Q97" t="inlineStr"/>
-      <c r="R97" t="inlineStr"/>
-      <c r="S97" t="inlineStr"/>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>2042600000965</t>
+        </is>
+      </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="S97" t="inlineStr">
+        <is>
+          <t>J1</t>
+        </is>
+      </c>
       <c r="T97" t="n">
         <v>0</v>
       </c>
@@ -9255,9 +10407,21 @@
       <c r="N98" t="inlineStr"/>
       <c r="O98" t="inlineStr"/>
       <c r="P98" t="inlineStr"/>
-      <c r="Q98" t="inlineStr"/>
-      <c r="R98" t="inlineStr"/>
-      <c r="S98" t="inlineStr"/>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>2042600000972</t>
+        </is>
+      </c>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>Cap</t>
+        </is>
+      </c>
+      <c r="S98" t="inlineStr">
+        <is>
+          <t>K1</t>
+        </is>
+      </c>
       <c r="T98" t="n">
         <v>0</v>
       </c>
@@ -9337,9 +10501,21 @@
       <c r="N99" t="inlineStr"/>
       <c r="O99" t="inlineStr"/>
       <c r="P99" t="inlineStr"/>
-      <c r="Q99" t="inlineStr"/>
-      <c r="R99" t="inlineStr"/>
-      <c r="S99" t="inlineStr"/>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>2042600000989</t>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>Tube</t>
+        </is>
+      </c>
+      <c r="S99" t="inlineStr">
+        <is>
+          <t>K2</t>
+        </is>
+      </c>
       <c r="T99" t="n">
         <v>0</v>
       </c>
@@ -9419,9 +10595,21 @@
       <c r="N100" t="inlineStr"/>
       <c r="O100" t="inlineStr"/>
       <c r="P100" t="inlineStr"/>
-      <c r="Q100" t="inlineStr"/>
-      <c r="R100" t="inlineStr"/>
-      <c r="S100" t="inlineStr"/>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>2042600000996</t>
+        </is>
+      </c>
+      <c r="R100" t="inlineStr">
+        <is>
+          <t>Tab</t>
+        </is>
+      </c>
+      <c r="S100" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
       <c r="T100" t="n">
         <v>0</v>
       </c>
@@ -9501,9 +10689,21 @@
       <c r="N101" t="inlineStr"/>
       <c r="O101" t="inlineStr"/>
       <c r="P101" t="inlineStr"/>
-      <c r="Q101" t="inlineStr"/>
-      <c r="R101" t="inlineStr"/>
-      <c r="S101" t="inlineStr"/>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>2042600001009</t>
+        </is>
+      </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>Tube</t>
+        </is>
+      </c>
+      <c r="S101" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
       <c r="T101" t="n">
         <v>0</v>
       </c>
@@ -9583,9 +10783,21 @@
       <c r="N102" t="inlineStr"/>
       <c r="O102" t="inlineStr"/>
       <c r="P102" t="inlineStr"/>
-      <c r="Q102" t="inlineStr"/>
-      <c r="R102" t="inlineStr"/>
-      <c r="S102" t="inlineStr"/>
+      <c r="Q102" t="inlineStr">
+        <is>
+          <t>2042600001016</t>
+        </is>
+      </c>
+      <c r="R102" t="inlineStr">
+        <is>
+          <t>Tube</t>
+        </is>
+      </c>
+      <c r="S102" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
       <c r="T102" t="n">
         <v>0</v>
       </c>
@@ -9665,9 +10877,21 @@
       <c r="N103" t="inlineStr"/>
       <c r="O103" t="inlineStr"/>
       <c r="P103" t="inlineStr"/>
-      <c r="Q103" t="inlineStr"/>
-      <c r="R103" t="inlineStr"/>
-      <c r="S103" t="inlineStr"/>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>2042600001023</t>
+        </is>
+      </c>
+      <c r="R103" t="inlineStr">
+        <is>
+          <t>Tube</t>
+        </is>
+      </c>
+      <c r="S103" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
       <c r="T103" t="n">
         <v>0</v>
       </c>
@@ -9747,9 +10971,21 @@
       <c r="N104" t="inlineStr"/>
       <c r="O104" t="inlineStr"/>
       <c r="P104" t="inlineStr"/>
-      <c r="Q104" t="inlineStr"/>
-      <c r="R104" t="inlineStr"/>
-      <c r="S104" t="inlineStr"/>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t>2042600001030</t>
+        </is>
+      </c>
+      <c r="R104" t="inlineStr">
+        <is>
+          <t>Btl</t>
+        </is>
+      </c>
+      <c r="S104" t="inlineStr">
+        <is>
+          <t>N1</t>
+        </is>
+      </c>
       <c r="T104" t="n">
         <v>0</v>
       </c>
@@ -9829,9 +11065,21 @@
       <c r="N105" t="inlineStr"/>
       <c r="O105" t="inlineStr"/>
       <c r="P105" t="inlineStr"/>
-      <c r="Q105" t="inlineStr"/>
-      <c r="R105" t="inlineStr"/>
-      <c r="S105" t="inlineStr"/>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t>2042600001047</t>
+        </is>
+      </c>
+      <c r="R105" t="inlineStr">
+        <is>
+          <t>Btl</t>
+        </is>
+      </c>
+      <c r="S105" t="inlineStr">
+        <is>
+          <t>N2</t>
+        </is>
+      </c>
       <c r="T105" t="n">
         <v>0</v>
       </c>
@@ -9911,9 +11159,21 @@
       <c r="N106" t="inlineStr"/>
       <c r="O106" t="inlineStr"/>
       <c r="P106" t="inlineStr"/>
-      <c r="Q106" t="inlineStr"/>
-      <c r="R106" t="inlineStr"/>
-      <c r="S106" t="inlineStr"/>
+      <c r="Q106" t="inlineStr">
+        <is>
+          <t>2042600001054</t>
+        </is>
+      </c>
+      <c r="R106" t="inlineStr">
+        <is>
+          <t>Btl</t>
+        </is>
+      </c>
+      <c r="S106" t="inlineStr">
+        <is>
+          <t>O1</t>
+        </is>
+      </c>
       <c r="T106" t="n">
         <v>0</v>
       </c>
@@ -9993,9 +11253,21 @@
       <c r="N107" t="inlineStr"/>
       <c r="O107" t="inlineStr"/>
       <c r="P107" t="inlineStr"/>
-      <c r="Q107" t="inlineStr"/>
-      <c r="R107" t="inlineStr"/>
-      <c r="S107" t="inlineStr"/>
+      <c r="Q107" t="inlineStr">
+        <is>
+          <t>2042600001061</t>
+        </is>
+      </c>
+      <c r="R107" t="inlineStr">
+        <is>
+          <t>Btl</t>
+        </is>
+      </c>
+      <c r="S107" t="inlineStr">
+        <is>
+          <t>O2</t>
+        </is>
+      </c>
       <c r="T107" t="n">
         <v>0</v>
       </c>
@@ -10071,9 +11343,21 @@
       <c r="N108" t="inlineStr"/>
       <c r="O108" t="inlineStr"/>
       <c r="P108" t="inlineStr"/>
-      <c r="Q108" t="inlineStr"/>
-      <c r="R108" t="inlineStr"/>
-      <c r="S108" t="inlineStr"/>
+      <c r="Q108" t="inlineStr">
+        <is>
+          <t>2042600001078</t>
+        </is>
+      </c>
+      <c r="R108" t="inlineStr">
+        <is>
+          <t>Btl</t>
+        </is>
+      </c>
+      <c r="S108" t="inlineStr">
+        <is>
+          <t>O3</t>
+        </is>
+      </c>
       <c r="T108" t="n">
         <v>0</v>
       </c>
@@ -10153,9 +11437,21 @@
       <c r="N109" t="inlineStr"/>
       <c r="O109" t="inlineStr"/>
       <c r="P109" t="inlineStr"/>
-      <c r="Q109" t="inlineStr"/>
-      <c r="R109" t="inlineStr"/>
-      <c r="S109" t="inlineStr"/>
+      <c r="Q109" t="inlineStr">
+        <is>
+          <t>2042600001085</t>
+        </is>
+      </c>
+      <c r="R109" t="inlineStr">
+        <is>
+          <t>Btl</t>
+        </is>
+      </c>
+      <c r="S109" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
       <c r="T109" t="n">
         <v>0</v>
       </c>
@@ -10195,7 +11491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -10245,29 +11541,43 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Barcodes and rack are left empty: barcodes are best scanned from the pack in the product form.</t>
+          <t>BARCODES ARE DUMMY TOO: valid EAN-13 codes in the 2… range kept for in-store use, so they never clash with a real pack.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Where the company is blank, the maker was not certain; fill it in from the pack.</t>
+          <t>Replace them with the barcode printed on each pack (or scan it in the product form). Rack numbers are examples.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Medicines are set to 0% sales tax.</t>
+          <t>Price per kg is empty because these are all sold by the pack, not by weight.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Where the company is blank, the maker was not certain; fill it in from the pack.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>Medicines are set to 0% sales tax.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>To import: Backoffice &gt; Inventory &gt; Import from Excel &gt; choose this file. The "Products" sheet is read.</t>
         </is>

</xml_diff>